<commit_message>
chore: actualizar archivo Facturación EESS
</commit_message>
<xml_diff>
--- a/Facturación EESS.xlsx
+++ b/Facturación EESS.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3756" uniqueCount="2059">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3875" uniqueCount="2125">
   <si>
     <t>Línea de Crédito Zeppelin</t>
   </si>
@@ -12160,12 +12160,18 @@
     <t>Razón Social</t>
   </si>
   <si>
+    <t>Proyecto</t>
+  </si>
+  <si>
     <t>AlmagroNacional | AO S | Por Categoria | Propiedades</t>
   </si>
   <si>
     <t>Nacional | AO S | Por Categoria | Propiedades</t>
   </si>
   <si>
+    <t>Propiedades</t>
+  </si>
+  <si>
     <t>AlmagroNacional | AO S | Propiedades | Cuota impresiones</t>
   </si>
   <si>
@@ -12184,12 +12190,18 @@
     <t>Antofagasta | MR | Parque Brasil</t>
   </si>
   <si>
+    <t>Antofagasta</t>
+  </si>
+  <si>
     <t>AlmagroNacional | AO S | Por Categoria | Always On</t>
   </si>
   <si>
     <t>Nacional | AO S | Por Categoria | Always On</t>
   </si>
   <si>
+    <t>Genérico</t>
+  </si>
+  <si>
     <t>AlmagroNorte | AO S | Por Comuna | Antofagasta</t>
   </si>
   <si>
@@ -12202,48 +12214,72 @@
     <t>Santiago | AO S | Inversionistas 2</t>
   </si>
   <si>
+    <t>Inversionista</t>
+  </si>
+  <si>
     <t>AlmagroSantiago | AO S | Por Comuna | Las Condes</t>
   </si>
   <si>
     <t>Santiago | AO S | Por Comuna | Las Condes</t>
   </si>
   <si>
+    <t>Las Condes</t>
+  </si>
+  <si>
     <t>AlmagroSantiago | AO S | Por Comuna | Lo Barnechea | Los Cactus</t>
   </si>
   <si>
     <t>Santiago | AO S | Por Comuna | Lo Barnechea | Los Cactus</t>
   </si>
   <si>
+    <t>Lo Barnechea</t>
+  </si>
+  <si>
     <t>AlmagroSantiago | AO S | Por Comuna | Macul | 2</t>
   </si>
   <si>
     <t>Santiago | AO S | Por Comuna | Macul | 2</t>
   </si>
   <si>
+    <t>Macul</t>
+  </si>
+  <si>
     <t>AlmagroSantiago | AO S | Por Comuna | Nunoa #2</t>
   </si>
   <si>
     <t>Santiago | AO S | Por Comuna | Nunoa #2</t>
   </si>
   <si>
+    <t>Ñuñoa</t>
+  </si>
+  <si>
     <t>AlmagroSantiago | AO S | Por Comuna | Providencia</t>
   </si>
   <si>
     <t>Santiago | AO S | Por Comuna | Providencia</t>
   </si>
   <si>
+    <t>Providencia</t>
+  </si>
+  <si>
     <t>AlmagroSantiago | AO S | Por Comuna | Santiago Centro #2</t>
   </si>
   <si>
     <t>Santiago | AO S | Por Comuna | Santiago Centro #2</t>
   </si>
   <si>
+    <t>Santiago Centro</t>
+  </si>
+  <si>
     <t>AlmagroSantiago | AO S | Tudeptoestupie</t>
   </si>
   <si>
     <t>Santiago | AO S | Tudeptoestupie</t>
   </si>
   <si>
+    <t>PPP</t>
+  </si>
+  <si>
     <t>AlmagroSantiago | Demand Gen | Almagro District</t>
   </si>
   <si>
@@ -12280,12 +12316,18 @@
     <t>FB_Advantage_Almagro</t>
   </si>
   <si>
+    <t>AON</t>
+  </si>
+  <si>
     <t>AlmagroFB_Almagro_Patrocinado_Blog</t>
   </si>
   <si>
     <t>FB_Almagro_Patrocinado_Blog</t>
   </si>
   <si>
+    <t>Blog</t>
+  </si>
+  <si>
     <t>AlmagroFB_Almagro_TuDeptoEsTuPie</t>
   </si>
   <si>
@@ -12298,84 +12340,126 @@
     <t>FB_AOL_Antofagasta_Indico</t>
   </si>
   <si>
+    <t>Indico</t>
+  </si>
+  <si>
     <t>AlmagroFB_AOL_Antofagasta_ParqueBrasil</t>
   </si>
   <si>
     <t>FB_AOL_Antofagasta_ParqueBrasil</t>
   </si>
   <si>
+    <t>Parque Brasil</t>
+  </si>
+  <si>
     <t>AlmagroFB_AOL_Santiago_AlmagroDistrict</t>
   </si>
   <si>
     <t>FB_AOL_Santiago_AlmagroDistrict</t>
   </si>
   <si>
+    <t>Almagro District</t>
+  </si>
+  <si>
     <t>AlmagroFB_AOL_Santiago_AlmagroHub</t>
   </si>
   <si>
     <t>FB_AOL_Santiago_AlmagroHub</t>
   </si>
   <si>
+    <t>Almagro Hub</t>
+  </si>
+  <si>
     <t>AlmagroFB_AOL_Santiago_AlmagroPlus</t>
   </si>
   <si>
     <t>FB_AOL_Santiago_AlmagroPlus</t>
   </si>
   <si>
+    <t>Almagro Plus</t>
+  </si>
+  <si>
     <t>AlmagroFB_AOL_Santiago_Balance</t>
   </si>
   <si>
     <t>FB_AOL_Santiago_Balance</t>
   </si>
   <si>
+    <t>Balance</t>
+  </si>
+  <si>
     <t>AlmagroFB_AOL_Santiago_Carrera_IV</t>
   </si>
   <si>
     <t>FB_AOL_Santiago_Carrera_IV</t>
   </si>
   <si>
+    <t>Carrera 4</t>
+  </si>
+  <si>
     <t>AlmagroFB_AOL_Santiago_Insigne</t>
   </si>
   <si>
     <t>FB_AOL_Santiago_Insigne</t>
   </si>
   <si>
+    <t>Insigne</t>
+  </si>
+  <si>
     <t>AlmagroFB_AOL_Santiago_LosCactus</t>
   </si>
   <si>
     <t>FB_AOL_Santiago_LosCactus</t>
   </si>
   <si>
+    <t>Los Cactus</t>
+  </si>
+  <si>
     <t>AlmagroFB_AOL_Santiago_LyonBilbao</t>
   </si>
   <si>
     <t>FB_AOL_Santiago_LyonBilbao</t>
   </si>
   <si>
+    <t>Lyon Bilbao</t>
+  </si>
+  <si>
     <t>AlmagroFB_AOL_Santiago_PadreLePaige_Etapa2</t>
   </si>
   <si>
     <t>FB_AOL_Santiago_PadreLePaige_Etapa2</t>
   </si>
   <si>
+    <t>PLP 2</t>
+  </si>
+  <si>
     <t>AlmagroFB_AOL_Santiago_PadreLePaige</t>
   </si>
   <si>
     <t>FB_AOL_Santiago_PadreLePaige</t>
   </si>
   <si>
+    <t>PLP 1</t>
+  </si>
+  <si>
     <t>AlmagroFB_AOL_Santiago_Rengo</t>
   </si>
   <si>
     <t>FB_AOL_Santiago_Rengo</t>
   </si>
   <si>
+    <t>Rengo</t>
+  </si>
+  <si>
     <t>AlmagroFB_AOL_Santiago_SanEugenio</t>
   </si>
   <si>
     <t>FB_AOL_Santiago_SanEugenio</t>
   </si>
   <si>
+    <t>San Eugenio 2</t>
+  </si>
+  <si>
     <t>AlmagroFB_AOT_Antofagasta_ParqueBrasil</t>
   </si>
   <si>
@@ -12445,24 +12529,36 @@
     <t>Santiago | AO S | Por Comuna | Estacion Central #2</t>
   </si>
   <si>
+    <t>Estación Central</t>
+  </si>
+  <si>
     <t>PilaresSantiago | AO S | Por Comuna | Independencia</t>
   </si>
   <si>
     <t>Santiago | AO S | Por Comuna | Independencia</t>
   </si>
   <si>
+    <t>Independencia</t>
+  </si>
+  <si>
     <t>PilaresSantiago | AO S | Por Comuna | La Cisterna</t>
   </si>
   <si>
     <t>Santiago | AO S | Por Comuna | La Cisterna</t>
   </si>
   <si>
+    <t>La Cisterna</t>
+  </si>
+  <si>
     <t>PilaresSantiago | AO S | Por Comuna | La Florida</t>
   </si>
   <si>
     <t>Santiago | AO S | Por Comuna | La Florida</t>
   </si>
   <si>
+    <t>La Florida</t>
+  </si>
+  <si>
     <t>PilaresSantiago | AO S | Por Comuna | Ñuñoa #2</t>
   </si>
   <si>
@@ -12490,48 +12586,72 @@
     <t>FB_AOL_CondeMauleIII</t>
   </si>
   <si>
+    <t>Conde del Maule</t>
+  </si>
+  <si>
     <t>PilaresFB_AOL_EdificioNuble</t>
   </si>
   <si>
     <t>FB_AOL_EdificioNuble</t>
   </si>
   <si>
+    <t>Edificio Ñuble</t>
+  </si>
+  <si>
     <t>PilaresFB_AOL_Franklin</t>
   </si>
   <si>
     <t>FB_AOL_Franklin</t>
   </si>
   <si>
+    <t>Franklin</t>
+  </si>
+  <si>
     <t>PilaresFB_AOL_GuillermoMann</t>
   </si>
   <si>
     <t>FB_AOL_GuillermoMann</t>
   </si>
   <si>
+    <t>Guillermo Mann</t>
+  </si>
+  <si>
     <t>PilaresFB_AOL_LoOvalle_E2</t>
   </si>
   <si>
     <t>FB_AOL_LoOvalle_E2</t>
   </si>
   <si>
+    <t>Lo Ovalle</t>
+  </si>
+  <si>
     <t>PilaresFB_AOL_RodriguezVelasco</t>
   </si>
   <si>
     <t>FB_AOL_RodriguezVelasco</t>
   </si>
   <si>
+    <t>Rodriguez Velasco</t>
+  </si>
+  <si>
     <t>PilaresFB_AOL_SantosDumont</t>
   </si>
   <si>
     <t>FB_AOL_SantosDumont</t>
   </si>
   <si>
+    <t>Santos Dumont</t>
+  </si>
+  <si>
     <t>PilaresFB_AOL_VicunaMackenna7244</t>
   </si>
   <si>
     <t>FB_AOL_VicunaMackenna7244</t>
   </si>
   <si>
+    <t>Vicuña Mackenna 7244</t>
+  </si>
+  <si>
     <t>PilaresFB_AOT_CondeMauleIII</t>
   </si>
   <si>
@@ -12586,6 +12706,9 @@
     <t>Santiago | AO S | Por Comuna | Lampa</t>
   </si>
   <si>
+    <t>Lampa</t>
+  </si>
+  <si>
     <t>Socovesa SantiagoSantiago | AO S | Por Comuna | Macul #2</t>
   </si>
   <si>
@@ -12598,6 +12721,9 @@
     <t>Santiago | AO S | Por Comuna | Maipu V2</t>
   </si>
   <si>
+    <t>Maipú</t>
+  </si>
+  <si>
     <t>Socovesa SantiagoSantiago | AO S | Por Comuna | Ñuñoa #2</t>
   </si>
   <si>
@@ -12637,36 +12763,54 @@
     <t>FB_AOL_SantiagoMedio_Coipue</t>
   </si>
   <si>
+    <t>Coipue</t>
+  </si>
+  <si>
     <t>Socovesa SantiagoFB_AOL_SantiagoMedio_LasPalmas</t>
   </si>
   <si>
     <t>FB_AOL_SantiagoMedio_LasPalmas</t>
   </si>
   <si>
+    <t>Las Palmas</t>
+  </si>
+  <si>
     <t>Socovesa SantiagoFB_AOL_SantiagoMedio_LosCoihues</t>
   </si>
   <si>
     <t>FB_AOL_SantiagoMedio_LosCoihues</t>
   </si>
   <si>
+    <t>Los Coihues</t>
+  </si>
+  <si>
     <t>Socovesa SantiagoFB_AOL_SantiagoMedio_Marathon</t>
   </si>
   <si>
     <t>FB_AOL_SantiagoMedio_Marathon</t>
   </si>
   <si>
+    <t>Marathon</t>
+  </si>
+  <si>
     <t>Socovesa SantiagoFB_AOL_SantiagoMedio_Pajaritos</t>
   </si>
   <si>
     <t>FB_AOL_SantiagoMedio_Pajaritos</t>
   </si>
   <si>
+    <t>Pajaritos</t>
+  </si>
+  <si>
     <t>Socovesa SantiagoFB_AOL_SantiagoSubsidio_LasPataguas</t>
   </si>
   <si>
     <t>FB_AOL_SantiagoSubsidio_LasPataguas</t>
   </si>
   <si>
+    <t>Las Pataguas</t>
+  </si>
+  <si>
     <t>Socovesa SantiagoFB_AOT_SantiagoMedio_LosCoihues</t>
   </si>
   <si>
@@ -12715,12 +12859,18 @@
     <t>Centro Sur | AO S | Por Ciudad | Chillan 2</t>
   </si>
   <si>
+    <t>Chillán</t>
+  </si>
+  <si>
     <t>Socovesa SurCentro Sur | AO S | Por Ciudad | Los Angeles #2</t>
   </si>
   <si>
     <t>Centro Sur | AO S | Por Ciudad | Los Angeles #2</t>
   </si>
   <si>
+    <t>Los Ángeles</t>
+  </si>
+  <si>
     <t>Socovesa SurSur | AO S | Inversionistas</t>
   </si>
   <si>
@@ -12739,94 +12889,142 @@
     <t>Sur | AO S | Por Ciudad | Temuco</t>
   </si>
   <si>
+    <t>Temuco</t>
+  </si>
+  <si>
     <t>Socovesa SurSur | AO S | Valdivia</t>
   </si>
   <si>
     <t>Sur | AO S | Valdivia</t>
   </si>
   <si>
+    <t>Valdivia</t>
+  </si>
+  <si>
     <t>Socovesa SurSur Austral | AO S | Por Ciudad | Puerto Montt</t>
   </si>
   <si>
     <t>Sur Austral | AO S | Por Ciudad | Puerto Montt</t>
   </si>
   <si>
+    <t>Puerto Montt</t>
+  </si>
+  <si>
     <t>Socovesa SurSur Austral | AO S | Por Ciudad | Punta Arenas</t>
   </si>
   <si>
     <t>Sur Austral | AO S | Por Ciudad | Punta Arenas</t>
   </si>
   <si>
+    <t>Punta Arenas</t>
+  </si>
+  <si>
     <t>Socovesa SurFB_AOL_CentroSur_AltoMaderosll</t>
   </si>
   <si>
     <t>FB_AOL_CentroSur_AltoMaderosll</t>
   </si>
   <si>
+    <t>Alto Maderos</t>
+  </si>
+  <si>
     <t>Socovesa SurFB_AOL_CentroSur_ElAvellano_E2</t>
   </si>
   <si>
     <t>FB_AOL_CentroSur_ElAvellano_E2</t>
   </si>
   <si>
+    <t>Parque Avellanos</t>
+  </si>
+  <si>
     <t>Socovesa SurFB_AOL_CentroSur_NuevaToledo</t>
   </si>
   <si>
     <t>FB_AOL_CentroSur_NuevaToledo</t>
   </si>
   <si>
+    <t>Nueva Toledo</t>
+  </si>
+  <si>
     <t>Socovesa SurFB_AOL_CentroSur_PortaldelLibertadorVIII</t>
   </si>
   <si>
     <t>FB_AOL_CentroSur_PortaldelLibertadorVIII</t>
   </si>
   <si>
+    <t>PDL</t>
+  </si>
+  <si>
     <t>Socovesa SurFB_AOL_Sur_CasasEnElPortal</t>
   </si>
   <si>
     <t>FB_AOL_Sur_CasasEnElPortal</t>
   </si>
   <si>
+    <t>Casas en el Portal</t>
+  </si>
+  <si>
     <t>Socovesa SurFB_AOL_Sur_EdificioVertice</t>
   </si>
   <si>
     <t>FB_AOL_Sur_EdificioVertice</t>
   </si>
   <si>
+    <t>Edificio Vértice</t>
+  </si>
+  <si>
     <t>Socovesa SurFB_AOL_Sur_GarciaReyes</t>
   </si>
   <si>
     <t>FB_AOL_Sur_GarciaReyes</t>
   </si>
   <si>
+    <t>García Reyes</t>
+  </si>
+  <si>
     <t>Socovesa SurFB_AOL_Sur_ParqueOlimpia_O3</t>
   </si>
   <si>
     <t>FB_AOL_Sur_ParqueOlimpia_O3</t>
   </si>
   <si>
+    <t>O3</t>
+  </si>
+  <si>
     <t>Socovesa SurFB_AOL_SurAustral_PortalAustral</t>
   </si>
   <si>
     <t>FB_AOL_SurAustral_PortalAustral</t>
   </si>
   <si>
+    <t>Portal Austral</t>
+  </si>
+  <si>
     <t>Socovesa SurFB_AOL_SurAustral_ReservaMagallanes</t>
   </si>
   <si>
     <t>FB_AOL_SurAustral_ReservaMagallanes</t>
   </si>
   <si>
+    <t>Reserva Magallanes</t>
+  </si>
+  <si>
     <t>Socovesa SurFB_AOL_SurAustral_TerrazaMiradorII</t>
   </si>
   <si>
     <t>FB_AOL_SurAustral_TerrazaMiradorII</t>
   </si>
   <si>
+    <t>Terraza Mirador</t>
+  </si>
+  <si>
     <t>Socovesa SurFB_AOL_Sur_VistaNielol_N3</t>
   </si>
   <si>
     <t>FB_AOL_Sur_VistaNielol_N3</t>
+  </si>
+  <si>
+    <t>N3</t>
   </si>
   <si>
     <t>Socovesa SurFB_AOT_CentroSur_PortaldelLibertador</t>
@@ -37494,1657 +37692,2014 @@
       <c r="E3" s="6" t="s">
         <v>1825</v>
       </c>
+      <c r="F3" s="6" t="s">
+        <v>1826</v>
+      </c>
     </row>
     <row r="4">
       <c r="B4" s="6" t="s">
-        <v>1826</v>
+        <v>1827</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>1827</v>
+        <v>1828</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F4" s="6" t="s">
+        <v>1829</v>
+      </c>
     </row>
     <row r="5">
       <c r="B5" s="6" t="s">
-        <v>1828</v>
+        <v>1830</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>1829</v>
+        <v>1831</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F5" s="6" t="s">
+        <v>1829</v>
+      </c>
     </row>
     <row r="6">
       <c r="B6" s="6" t="s">
-        <v>1830</v>
+        <v>1832</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>1831</v>
+        <v>1833</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F6" s="6" t="s">
+        <v>1829</v>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="6" t="s">
-        <v>1832</v>
+        <v>1834</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>1833</v>
+        <v>1835</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F7" s="6" t="s">
+        <v>1836</v>
+      </c>
     </row>
     <row r="8">
       <c r="B8" s="6" t="s">
-        <v>1834</v>
+        <v>1837</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>1835</v>
+        <v>1838</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F8" s="6" t="s">
+        <v>1839</v>
+      </c>
     </row>
     <row r="9">
       <c r="B9" s="6" t="s">
-        <v>1836</v>
+        <v>1840</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>1837</v>
+        <v>1841</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F9" s="6" t="s">
+        <v>1836</v>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="6" t="s">
-        <v>1838</v>
+        <v>1842</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>1839</v>
+        <v>1843</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F10" s="6" t="s">
+        <v>1844</v>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="6" t="s">
-        <v>1840</v>
+        <v>1845</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>1841</v>
+        <v>1846</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F11" s="6" t="s">
+        <v>1847</v>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="6" t="s">
-        <v>1842</v>
+        <v>1848</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>1843</v>
+        <v>1849</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F12" s="6" t="s">
+        <v>1850</v>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="6" t="s">
-        <v>1844</v>
+        <v>1851</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>1845</v>
+        <v>1852</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F13" s="6" t="s">
+        <v>1853</v>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="6" t="s">
-        <v>1846</v>
+        <v>1854</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>1847</v>
+        <v>1855</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F14" s="6" t="s">
+        <v>1856</v>
+      </c>
     </row>
     <row r="15">
       <c r="B15" s="6" t="s">
-        <v>1848</v>
+        <v>1857</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>1849</v>
+        <v>1858</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F15" s="6" t="s">
+        <v>1859</v>
+      </c>
     </row>
     <row r="16">
       <c r="B16" s="6" t="s">
-        <v>1850</v>
+        <v>1860</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>1851</v>
+        <v>1861</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F16" s="6" t="s">
+        <v>1862</v>
+      </c>
     </row>
     <row r="17">
       <c r="B17" s="6" t="s">
-        <v>1852</v>
+        <v>1863</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>1853</v>
+        <v>1864</v>
       </c>
       <c r="E17" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F17" s="6" t="s">
+        <v>1865</v>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="6" t="s">
-        <v>1854</v>
+        <v>1866</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>1855</v>
+        <v>1867</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>1810</v>
       </c>
+      <c r="F18" s="6" t="s">
+        <v>1847</v>
+      </c>
     </row>
     <row r="19">
       <c r="B19" s="6" t="s">
-        <v>1856</v>
+        <v>1868</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>1857</v>
+        <v>1869</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>1810</v>
       </c>
+      <c r="F19" s="6" t="s">
+        <v>1847</v>
+      </c>
     </row>
     <row r="20">
       <c r="B20" s="6" t="s">
-        <v>1858</v>
+        <v>1870</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>1859</v>
+        <v>1871</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F20" s="6" t="s">
+        <v>1853</v>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="6" t="s">
-        <v>1860</v>
+        <v>1872</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>1861</v>
+        <v>1873</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F21" s="6" t="s">
+        <v>1856</v>
+      </c>
     </row>
     <row r="22">
       <c r="B22" s="6" t="s">
-        <v>1862</v>
+        <v>1874</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>1863</v>
+        <v>1875</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>1811</v>
       </c>
+      <c r="F22" s="6" t="s">
+        <v>1859</v>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="6" t="s">
-        <v>1864</v>
+        <v>1876</v>
       </c>
       <c r="C23" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>1865</v>
+        <v>1877</v>
       </c>
       <c r="E23" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F23" s="6" t="s">
+        <v>1878</v>
+      </c>
     </row>
     <row r="24">
       <c r="B24" s="6" t="s">
-        <v>1866</v>
+        <v>1879</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>1867</v>
+        <v>1880</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F24" s="6" t="s">
+        <v>1881</v>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="6" t="s">
-        <v>1868</v>
+        <v>1882</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>1869</v>
+        <v>1883</v>
       </c>
       <c r="E25" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F25" s="6" t="s">
+        <v>1865</v>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="6" t="s">
-        <v>1870</v>
+        <v>1884</v>
       </c>
       <c r="C26" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>1871</v>
+        <v>1885</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F26" s="6" t="s">
+        <v>1886</v>
+      </c>
     </row>
     <row r="27">
       <c r="B27" s="6" t="s">
-        <v>1872</v>
+        <v>1887</v>
       </c>
       <c r="C27" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>1873</v>
+        <v>1888</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F27" s="6" t="s">
+        <v>1889</v>
+      </c>
     </row>
     <row r="28">
       <c r="B28" s="6" t="s">
-        <v>1874</v>
+        <v>1890</v>
       </c>
       <c r="C28" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>1875</v>
+        <v>1891</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>1810</v>
       </c>
+      <c r="F28" s="6" t="s">
+        <v>1892</v>
+      </c>
     </row>
     <row r="29">
       <c r="B29" s="6" t="s">
-        <v>1876</v>
+        <v>1893</v>
       </c>
       <c r="C29" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>1877</v>
+        <v>1894</v>
       </c>
       <c r="E29" s="6" t="s">
         <v>1811</v>
       </c>
+      <c r="F29" s="6" t="s">
+        <v>1895</v>
+      </c>
     </row>
     <row r="30">
       <c r="B30" s="6" t="s">
-        <v>1878</v>
+        <v>1896</v>
       </c>
       <c r="C30" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>1879</v>
+        <v>1897</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F30" s="6" t="s">
+        <v>1898</v>
+      </c>
     </row>
     <row r="31">
       <c r="B31" s="6" t="s">
-        <v>1880</v>
+        <v>1899</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>1881</v>
+        <v>1900</v>
       </c>
       <c r="E31" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F31" s="6" t="s">
+        <v>1901</v>
+      </c>
     </row>
     <row r="32">
       <c r="B32" s="6" t="s">
-        <v>1882</v>
+        <v>1902</v>
       </c>
       <c r="C32" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>1883</v>
+        <v>1903</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F32" s="6" t="s">
+        <v>1904</v>
+      </c>
     </row>
     <row r="33">
       <c r="B33" s="6" t="s">
-        <v>1884</v>
+        <v>1905</v>
       </c>
       <c r="C33" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>1885</v>
+        <v>1906</v>
       </c>
       <c r="E33" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F33" s="6" t="s">
+        <v>1907</v>
+      </c>
     </row>
     <row r="34">
       <c r="B34" s="6" t="s">
-        <v>1886</v>
+        <v>1908</v>
       </c>
       <c r="C34" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>1887</v>
+        <v>1909</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F34" s="6" t="s">
+        <v>1910</v>
+      </c>
     </row>
     <row r="35">
       <c r="B35" s="6" t="s">
-        <v>1888</v>
+        <v>1911</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>1889</v>
+        <v>1912</v>
       </c>
       <c r="E35" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F35" s="6" t="s">
+        <v>1913</v>
+      </c>
     </row>
     <row r="36">
       <c r="B36" s="6" t="s">
-        <v>1890</v>
+        <v>1914</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>1891</v>
+        <v>1915</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>1811</v>
       </c>
+      <c r="F36" s="6" t="s">
+        <v>1916</v>
+      </c>
     </row>
     <row r="37">
       <c r="B37" s="6" t="s">
-        <v>1892</v>
+        <v>1917</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>1893</v>
+        <v>1918</v>
       </c>
       <c r="E37" s="6" t="s">
         <v>1811</v>
       </c>
+      <c r="F37" s="6" t="s">
+        <v>1919</v>
+      </c>
     </row>
     <row r="38">
       <c r="B38" s="6" t="s">
-        <v>1894</v>
+        <v>1920</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>1895</v>
+        <v>1921</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>1811</v>
       </c>
+      <c r="F38" s="6" t="s">
+        <v>1922</v>
+      </c>
     </row>
     <row r="39">
       <c r="B39" s="6" t="s">
-        <v>1896</v>
+        <v>1923</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>1897</v>
+        <v>1924</v>
       </c>
       <c r="E39" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F39" s="6" t="s">
+        <v>1925</v>
+      </c>
     </row>
     <row r="40">
       <c r="B40" s="6" t="s">
-        <v>1898</v>
+        <v>1926</v>
       </c>
       <c r="C40" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>1899</v>
+        <v>1927</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F40" s="6" t="s">
+        <v>1889</v>
+      </c>
     </row>
     <row r="41">
       <c r="B41" s="6" t="s">
-        <v>1900</v>
+        <v>1928</v>
       </c>
       <c r="C41" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>1901</v>
+        <v>1929</v>
       </c>
       <c r="E41" s="6" t="s">
         <v>1810</v>
       </c>
+      <c r="F41" s="6" t="s">
+        <v>1892</v>
+      </c>
     </row>
     <row r="42">
       <c r="B42" s="6" t="s">
-        <v>1902</v>
+        <v>1930</v>
       </c>
       <c r="C42" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>1903</v>
+        <v>1931</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F42" s="6" t="s">
+        <v>1898</v>
+      </c>
     </row>
     <row r="43">
       <c r="B43" s="6" t="s">
-        <v>1904</v>
+        <v>1932</v>
       </c>
       <c r="C43" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>1905</v>
+        <v>1933</v>
       </c>
       <c r="E43" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F43" s="6" t="s">
+        <v>1901</v>
+      </c>
     </row>
     <row r="44">
       <c r="B44" s="6" t="s">
-        <v>1906</v>
+        <v>1934</v>
       </c>
       <c r="C44" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>1907</v>
+        <v>1935</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F44" s="6" t="s">
+        <v>1907</v>
+      </c>
     </row>
     <row r="45">
       <c r="B45" s="6" t="s">
-        <v>1908</v>
+        <v>1936</v>
       </c>
       <c r="C45" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>1909</v>
+        <v>1937</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>1811</v>
       </c>
+      <c r="F45" s="6" t="s">
+        <v>1922</v>
+      </c>
     </row>
     <row r="46">
       <c r="B46" s="6" t="s">
-        <v>1910</v>
+        <v>1938</v>
       </c>
       <c r="C46" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>1911</v>
+        <v>1939</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F46" s="6" t="s">
+        <v>1878</v>
+      </c>
     </row>
     <row r="47">
       <c r="B47" s="6" t="s">
-        <v>1912</v>
+        <v>1940</v>
       </c>
       <c r="C47" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>1913</v>
+        <v>1941</v>
       </c>
       <c r="E47" s="6" t="s">
         <v>1809</v>
       </c>
+      <c r="F47" s="6" t="s">
+        <v>1802</v>
+      </c>
     </row>
     <row r="48">
       <c r="B48" s="6" t="s">
-        <v>1914</v>
+        <v>1942</v>
       </c>
       <c r="C48" s="6" t="s">
         <v>8</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>1915</v>
+        <v>1943</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>1811</v>
       </c>
+      <c r="F48" s="6" t="s">
+        <v>1916</v>
+      </c>
     </row>
     <row r="49">
       <c r="B49" s="6" t="s">
-        <v>1916</v>
+        <v>1944</v>
       </c>
       <c r="C49" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>1917</v>
+        <v>1945</v>
       </c>
       <c r="E49" s="6" t="s">
         <v>1813</v>
       </c>
+      <c r="F49" s="6" t="s">
+        <v>1839</v>
+      </c>
     </row>
     <row r="50">
       <c r="B50" s="6" t="s">
-        <v>1918</v>
+        <v>1946</v>
       </c>
       <c r="C50" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>1839</v>
+        <v>1843</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>1813</v>
       </c>
+      <c r="F50" s="6" t="s">
+        <v>1844</v>
+      </c>
     </row>
     <row r="51">
       <c r="B51" s="6" t="s">
-        <v>1919</v>
+        <v>1947</v>
       </c>
       <c r="C51" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>1920</v>
+        <v>1948</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>1814</v>
       </c>
+      <c r="F51" s="6" t="s">
+        <v>1949</v>
+      </c>
     </row>
     <row r="52">
       <c r="B52" s="6" t="s">
-        <v>1921</v>
+        <v>1950</v>
       </c>
       <c r="C52" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>1922</v>
+        <v>1951</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>1814</v>
       </c>
+      <c r="F52" s="6" t="s">
+        <v>1952</v>
+      </c>
     </row>
     <row r="53">
       <c r="B53" s="6" t="s">
-        <v>1923</v>
+        <v>1953</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>1924</v>
+        <v>1954</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>1814</v>
       </c>
+      <c r="F53" s="6" t="s">
+        <v>1955</v>
+      </c>
     </row>
     <row r="54">
       <c r="B54" s="6" t="s">
-        <v>1925</v>
+        <v>1956</v>
       </c>
       <c r="C54" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>1926</v>
+        <v>1957</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>1813</v>
       </c>
+      <c r="F54" s="6" t="s">
+        <v>1958</v>
+      </c>
     </row>
     <row r="55">
       <c r="B55" s="6" t="s">
-        <v>1927</v>
+        <v>1959</v>
       </c>
       <c r="C55" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>1928</v>
+        <v>1960</v>
       </c>
       <c r="E55" s="6" t="s">
         <v>1813</v>
       </c>
+      <c r="F55" s="6" t="s">
+        <v>1856</v>
+      </c>
     </row>
     <row r="56">
       <c r="B56" s="6" t="s">
-        <v>1929</v>
+        <v>1961</v>
       </c>
       <c r="C56" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>1851</v>
+        <v>1861</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>1814</v>
       </c>
+      <c r="F56" s="6" t="s">
+        <v>1862</v>
+      </c>
     </row>
     <row r="57">
       <c r="B57" s="6" t="s">
-        <v>1930</v>
+        <v>1962</v>
       </c>
       <c r="C57" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>1931</v>
+        <v>1963</v>
       </c>
       <c r="E57" s="6" t="s">
         <v>1814</v>
       </c>
+      <c r="F57" s="6" t="s">
+        <v>1949</v>
+      </c>
     </row>
     <row r="58">
       <c r="B58" s="6" t="s">
-        <v>1932</v>
+        <v>1964</v>
       </c>
       <c r="C58" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>1933</v>
+        <v>1965</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>1814</v>
       </c>
+      <c r="F58" s="6" t="s">
+        <v>1952</v>
+      </c>
     </row>
     <row r="59">
       <c r="B59" s="6" t="s">
-        <v>1934</v>
+        <v>1966</v>
       </c>
       <c r="C59" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>1935</v>
+        <v>1967</v>
       </c>
       <c r="E59" s="6" t="s">
         <v>1814</v>
       </c>
+      <c r="F59" s="6" t="s">
+        <v>1968</v>
+      </c>
     </row>
     <row r="60">
       <c r="B60" s="6" t="s">
-        <v>1936</v>
+        <v>1969</v>
       </c>
       <c r="C60" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>1937</v>
+        <v>1970</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>1814</v>
       </c>
+      <c r="F60" s="6" t="s">
+        <v>1971</v>
+      </c>
     </row>
     <row r="61">
       <c r="B61" s="6" t="s">
-        <v>1938</v>
+        <v>1972</v>
       </c>
       <c r="C61" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>1939</v>
+        <v>1973</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>1811</v>
       </c>
+      <c r="F61" s="6" t="s">
+        <v>1974</v>
+      </c>
     </row>
     <row r="62">
       <c r="B62" s="6" t="s">
-        <v>1940</v>
+        <v>1975</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>1941</v>
+        <v>1976</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>1813</v>
       </c>
+      <c r="F62" s="6" t="s">
+        <v>1977</v>
+      </c>
     </row>
     <row r="63">
       <c r="B63" s="6" t="s">
-        <v>1942</v>
+        <v>1978</v>
       </c>
       <c r="C63" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>1943</v>
+        <v>1979</v>
       </c>
       <c r="E63" s="6" t="s">
         <v>1814</v>
       </c>
+      <c r="F63" s="6" t="s">
+        <v>1980</v>
+      </c>
     </row>
     <row r="64">
       <c r="B64" s="6" t="s">
-        <v>1944</v>
+        <v>1981</v>
       </c>
       <c r="C64" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>1945</v>
+        <v>1982</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>1813</v>
       </c>
+      <c r="F64" s="6" t="s">
+        <v>1983</v>
+      </c>
     </row>
     <row r="65">
       <c r="B65" s="6" t="s">
-        <v>1946</v>
+        <v>1984</v>
       </c>
       <c r="C65" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>1947</v>
+        <v>1985</v>
       </c>
       <c r="E65" s="6" t="s">
         <v>1814</v>
       </c>
+      <c r="F65" s="6" t="s">
+        <v>1986</v>
+      </c>
     </row>
     <row r="66">
       <c r="B66" s="6" t="s">
-        <v>1948</v>
+        <v>1987</v>
       </c>
       <c r="C66" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>1949</v>
+        <v>1988</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>1813</v>
       </c>
+      <c r="F66" s="6" t="s">
+        <v>1989</v>
+      </c>
     </row>
     <row r="67">
       <c r="B67" s="6" t="s">
-        <v>1950</v>
+        <v>1990</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>1951</v>
+        <v>1991</v>
       </c>
       <c r="E67" s="6" t="s">
         <v>1814</v>
       </c>
+      <c r="F67" s="6" t="s">
+        <v>1968</v>
+      </c>
     </row>
     <row r="68">
       <c r="B68" s="6" t="s">
-        <v>1952</v>
+        <v>1992</v>
       </c>
       <c r="C68" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>1953</v>
+        <v>1993</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>1811</v>
       </c>
+      <c r="F68" s="6" t="s">
+        <v>1974</v>
+      </c>
     </row>
     <row r="69">
       <c r="B69" s="6" t="s">
-        <v>1954</v>
+        <v>1994</v>
       </c>
       <c r="C69" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>1955</v>
+        <v>1995</v>
       </c>
       <c r="E69" s="6" t="s">
         <v>1814</v>
       </c>
+      <c r="F69" s="6" t="s">
+        <v>1986</v>
+      </c>
     </row>
     <row r="70">
       <c r="B70" s="6" t="s">
-        <v>1956</v>
+        <v>1996</v>
       </c>
       <c r="C70" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>1957</v>
+        <v>1997</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>1813</v>
       </c>
+      <c r="F70" s="6" t="s">
+        <v>1878</v>
+      </c>
     </row>
     <row r="71">
       <c r="B71" s="6" t="s">
-        <v>1958</v>
+        <v>1998</v>
       </c>
       <c r="C71" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>1959</v>
+        <v>1999</v>
       </c>
       <c r="E71" s="6" t="s">
         <v>1813</v>
       </c>
+      <c r="F71" s="6" t="s">
+        <v>1802</v>
+      </c>
     </row>
     <row r="72">
       <c r="B72" s="6" t="s">
-        <v>1960</v>
+        <v>2000</v>
       </c>
       <c r="C72" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>1961</v>
+        <v>2001</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>1813</v>
       </c>
+      <c r="F72" s="6" t="s">
+        <v>1844</v>
+      </c>
     </row>
     <row r="73">
       <c r="B73" s="6" t="s">
-        <v>1962</v>
+        <v>2002</v>
       </c>
       <c r="C73" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>1963</v>
+        <v>2003</v>
       </c>
       <c r="E73" s="6" t="s">
         <v>1813</v>
       </c>
+      <c r="F73" s="6" t="s">
+        <v>1844</v>
+      </c>
     </row>
     <row r="74">
       <c r="B74" s="6" t="s">
-        <v>1964</v>
+        <v>2004</v>
       </c>
       <c r="C74" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>1965</v>
+        <v>2005</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>1816</v>
       </c>
+      <c r="F74" s="6" t="s">
+        <v>1839</v>
+      </c>
     </row>
     <row r="75">
       <c r="B75" s="6" t="s">
-        <v>1966</v>
+        <v>2006</v>
       </c>
       <c r="C75" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>1967</v>
+        <v>2007</v>
       </c>
       <c r="E75" s="6" t="s">
         <v>1817</v>
       </c>
+      <c r="F75" s="6" t="s">
+        <v>2008</v>
+      </c>
     </row>
     <row r="76">
       <c r="B76" s="6" t="s">
-        <v>1968</v>
+        <v>2009</v>
       </c>
       <c r="C76" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>1969</v>
+        <v>2010</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>1818</v>
       </c>
+      <c r="F76" s="6" t="s">
+        <v>1853</v>
+      </c>
     </row>
     <row r="77">
       <c r="B77" s="6" t="s">
-        <v>1970</v>
+        <v>2011</v>
       </c>
       <c r="C77" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>1971</v>
+        <v>2012</v>
       </c>
       <c r="E77" s="6" t="s">
         <v>1819</v>
       </c>
+      <c r="F77" s="6" t="s">
+        <v>2013</v>
+      </c>
     </row>
     <row r="78">
       <c r="B78" s="6" t="s">
-        <v>1972</v>
+        <v>2014</v>
       </c>
       <c r="C78" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>1928</v>
+        <v>1960</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>1819</v>
       </c>
+      <c r="F78" s="6" t="s">
+        <v>1856</v>
+      </c>
     </row>
     <row r="79">
       <c r="B79" s="6" t="s">
-        <v>1973</v>
+        <v>2015</v>
       </c>
       <c r="C79" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>1974</v>
+        <v>2016</v>
       </c>
       <c r="E79" s="6" t="s">
         <v>1817</v>
       </c>
+      <c r="F79" s="6" t="s">
+        <v>2008</v>
+      </c>
     </row>
     <row r="80">
       <c r="B80" s="6" t="s">
-        <v>1975</v>
+        <v>2017</v>
       </c>
       <c r="C80" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>1976</v>
+        <v>2018</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>1820</v>
       </c>
+      <c r="F80" s="6" t="s">
+        <v>1853</v>
+      </c>
     </row>
     <row r="81">
       <c r="B81" s="6" t="s">
-        <v>1977</v>
+        <v>2019</v>
       </c>
       <c r="C81" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>1978</v>
+        <v>2020</v>
       </c>
       <c r="E81" s="6" t="s">
         <v>1817</v>
       </c>
+      <c r="F81" s="6" t="s">
+        <v>2008</v>
+      </c>
     </row>
     <row r="82">
       <c r="B82" s="6" t="s">
-        <v>1979</v>
+        <v>2021</v>
       </c>
       <c r="C82" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>1980</v>
+        <v>2022</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>1819</v>
       </c>
+      <c r="F82" s="6" t="s">
+        <v>2013</v>
+      </c>
     </row>
     <row r="83">
       <c r="B83" s="6" t="s">
-        <v>1981</v>
+        <v>2023</v>
       </c>
       <c r="C83" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>1982</v>
+        <v>2024</v>
       </c>
       <c r="E83" s="6" t="s">
         <v>1813</v>
       </c>
+      <c r="F83" s="6" t="s">
+        <v>1856</v>
+      </c>
     </row>
     <row r="84">
       <c r="B84" s="6" t="s">
-        <v>1983</v>
+        <v>2025</v>
       </c>
       <c r="C84" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>1984</v>
+        <v>2026</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>1820</v>
       </c>
+      <c r="F84" s="6" t="s">
+        <v>2027</v>
+      </c>
     </row>
     <row r="85">
       <c r="B85" s="6" t="s">
-        <v>1985</v>
+        <v>2028</v>
       </c>
       <c r="C85" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>1986</v>
+        <v>2029</v>
       </c>
       <c r="E85" s="6" t="s">
         <v>1818</v>
       </c>
+      <c r="F85" s="6" t="s">
+        <v>2030</v>
+      </c>
     </row>
     <row r="86">
       <c r="B86" s="6" t="s">
-        <v>1987</v>
+        <v>2031</v>
       </c>
       <c r="C86" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>1988</v>
+        <v>2032</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>1817</v>
       </c>
+      <c r="F86" s="6" t="s">
+        <v>2033</v>
+      </c>
     </row>
     <row r="87">
       <c r="B87" s="6" t="s">
-        <v>1989</v>
+        <v>2034</v>
       </c>
       <c r="C87" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>1990</v>
+        <v>2035</v>
       </c>
       <c r="E87" s="6" t="s">
         <v>1813</v>
       </c>
+      <c r="F87" s="6" t="s">
+        <v>2036</v>
+      </c>
     </row>
     <row r="88">
       <c r="B88" s="6" t="s">
-        <v>1991</v>
+        <v>2037</v>
       </c>
       <c r="C88" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>1992</v>
+        <v>2038</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>1819</v>
       </c>
+      <c r="F88" s="6" t="s">
+        <v>2039</v>
+      </c>
     </row>
     <row r="89">
       <c r="B89" s="6" t="s">
-        <v>1993</v>
+        <v>2040</v>
       </c>
       <c r="C89" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D89" s="6" t="s">
-        <v>1994</v>
+        <v>2041</v>
       </c>
       <c r="E89" s="6" t="s">
         <v>1817</v>
       </c>
+      <c r="F89" s="6" t="s">
+        <v>2042</v>
+      </c>
     </row>
     <row r="90">
       <c r="B90" s="6" t="s">
-        <v>1995</v>
+        <v>2043</v>
       </c>
       <c r="C90" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>1996</v>
+        <v>2044</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>1817</v>
       </c>
+      <c r="F90" s="6" t="s">
+        <v>2033</v>
+      </c>
     </row>
     <row r="91">
       <c r="B91" s="6" t="s">
-        <v>1997</v>
+        <v>2045</v>
       </c>
       <c r="C91" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>1998</v>
+        <v>2046</v>
       </c>
       <c r="E91" s="6" t="s">
         <v>1813</v>
       </c>
+      <c r="F91" s="6" t="s">
+        <v>2036</v>
+      </c>
     </row>
     <row r="92">
       <c r="B92" s="6" t="s">
-        <v>1999</v>
+        <v>2047</v>
       </c>
       <c r="C92" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D92" s="6" t="s">
-        <v>2000</v>
+        <v>2048</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>1819</v>
       </c>
+      <c r="F92" s="6" t="s">
+        <v>2039</v>
+      </c>
     </row>
     <row r="93">
       <c r="B93" s="6" t="s">
-        <v>2001</v>
+        <v>2049</v>
       </c>
       <c r="C93" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D93" s="6" t="s">
-        <v>2002</v>
+        <v>2050</v>
       </c>
       <c r="E93" s="6" t="s">
         <v>1817</v>
       </c>
+      <c r="F93" s="6" t="s">
+        <v>2042</v>
+      </c>
     </row>
     <row r="94">
       <c r="B94" s="6" t="s">
-        <v>2003</v>
+        <v>2051</v>
       </c>
       <c r="C94" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D94" s="6" t="s">
-        <v>2004</v>
+        <v>2052</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>1816</v>
       </c>
+      <c r="F94" s="6" t="s">
+        <v>1878</v>
+      </c>
     </row>
     <row r="95">
       <c r="B95" s="6" t="s">
-        <v>2005</v>
+        <v>2053</v>
       </c>
       <c r="C95" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D95" s="6" t="s">
-        <v>2006</v>
+        <v>2054</v>
       </c>
       <c r="E95" s="6" t="s">
         <v>1816</v>
       </c>
+      <c r="F95" s="6" t="s">
+        <v>1802</v>
+      </c>
     </row>
     <row r="96">
       <c r="B96" s="6" t="s">
-        <v>2007</v>
+        <v>2055</v>
       </c>
       <c r="C96" s="6" t="s">
         <v>1815</v>
       </c>
       <c r="D96" s="6" t="s">
-        <v>2008</v>
+        <v>2056</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>1816</v>
       </c>
+      <c r="F96" s="6" t="s">
+        <v>1802</v>
+      </c>
     </row>
     <row r="97">
       <c r="B97" s="6" t="s">
-        <v>2009</v>
+        <v>2057</v>
       </c>
       <c r="C97" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D97" s="6" t="s">
-        <v>2010</v>
+        <v>2058</v>
       </c>
       <c r="E97" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F97" s="6" t="s">
+        <v>2059</v>
+      </c>
     </row>
     <row r="98">
       <c r="B98" s="6" t="s">
-        <v>2011</v>
+        <v>2060</v>
       </c>
       <c r="C98" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D98" s="6" t="s">
-        <v>2012</v>
+        <v>2061</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F98" s="6" t="s">
+        <v>2062</v>
+      </c>
     </row>
     <row r="99">
       <c r="B99" s="6" t="s">
-        <v>2013</v>
+        <v>2063</v>
       </c>
       <c r="C99" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D99" s="6" t="s">
-        <v>2014</v>
+        <v>2064</v>
       </c>
       <c r="E99" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F99" s="6" t="s">
+        <v>1844</v>
+      </c>
     </row>
     <row r="100">
       <c r="B100" s="6" t="s">
-        <v>2015</v>
+        <v>2065</v>
       </c>
       <c r="C100" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D100" s="6" t="s">
-        <v>2016</v>
+        <v>2066</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F100" s="6" t="s">
+        <v>1839</v>
+      </c>
     </row>
     <row r="101">
       <c r="B101" s="6" t="s">
-        <v>2017</v>
+        <v>2067</v>
       </c>
       <c r="C101" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D101" s="6" t="s">
-        <v>2018</v>
+        <v>2068</v>
       </c>
       <c r="E101" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F101" s="6" t="s">
+        <v>2069</v>
+      </c>
     </row>
     <row r="102">
       <c r="B102" s="6" t="s">
-        <v>2019</v>
+        <v>2070</v>
       </c>
       <c r="C102" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D102" s="6" t="s">
-        <v>2020</v>
+        <v>2071</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F102" s="6" t="s">
+        <v>2072</v>
+      </c>
     </row>
     <row r="103">
       <c r="B103" s="6" t="s">
-        <v>2021</v>
+        <v>2073</v>
       </c>
       <c r="C103" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D103" s="6" t="s">
-        <v>2022</v>
+        <v>2074</v>
       </c>
       <c r="E103" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F103" s="6" t="s">
+        <v>2075</v>
+      </c>
     </row>
     <row r="104">
       <c r="B104" s="6" t="s">
-        <v>2023</v>
+        <v>2076</v>
       </c>
       <c r="C104" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D104" s="6" t="s">
-        <v>2024</v>
+        <v>2077</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F104" s="6" t="s">
+        <v>2078</v>
+      </c>
     </row>
     <row r="105">
       <c r="B105" s="6" t="s">
-        <v>2025</v>
+        <v>2079</v>
       </c>
       <c r="C105" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D105" s="6" t="s">
-        <v>2026</v>
+        <v>2080</v>
       </c>
       <c r="E105" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F105" s="6" t="s">
+        <v>2081</v>
+      </c>
     </row>
     <row r="106">
       <c r="B106" s="6" t="s">
-        <v>2027</v>
+        <v>2082</v>
       </c>
       <c r="C106" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D106" s="6" t="s">
-        <v>2028</v>
+        <v>2083</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F106" s="6" t="s">
+        <v>2084</v>
+      </c>
     </row>
     <row r="107">
       <c r="B107" s="6" t="s">
-        <v>2029</v>
+        <v>2085</v>
       </c>
       <c r="C107" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D107" s="6" t="s">
-        <v>2030</v>
+        <v>2086</v>
       </c>
       <c r="E107" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F107" s="6" t="s">
+        <v>2087</v>
+      </c>
     </row>
     <row r="108">
       <c r="B108" s="6" t="s">
-        <v>2031</v>
+        <v>2088</v>
       </c>
       <c r="C108" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D108" s="6" t="s">
-        <v>2032</v>
+        <v>2089</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F108" s="6" t="s">
+        <v>2090</v>
+      </c>
     </row>
     <row r="109">
       <c r="B109" s="6" t="s">
-        <v>2033</v>
+        <v>2091</v>
       </c>
       <c r="C109" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D109" s="6" t="s">
-        <v>2034</v>
+        <v>2092</v>
       </c>
       <c r="E109" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F109" s="6" t="s">
+        <v>2093</v>
+      </c>
     </row>
     <row r="110">
       <c r="B110" s="6" t="s">
-        <v>2035</v>
+        <v>2094</v>
       </c>
       <c r="C110" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D110" s="6" t="s">
-        <v>2036</v>
+        <v>2095</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F110" s="6" t="s">
+        <v>2096</v>
+      </c>
     </row>
     <row r="111">
       <c r="B111" s="6" t="s">
-        <v>2037</v>
+        <v>2097</v>
       </c>
       <c r="C111" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D111" s="6" t="s">
-        <v>2038</v>
+        <v>2098</v>
       </c>
       <c r="E111" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F111" s="6" t="s">
+        <v>2099</v>
+      </c>
     </row>
     <row r="112">
       <c r="B112" s="6" t="s">
-        <v>2039</v>
+        <v>2100</v>
       </c>
       <c r="C112" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D112" s="6" t="s">
-        <v>2040</v>
+        <v>2101</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F112" s="6" t="s">
+        <v>2102</v>
+      </c>
     </row>
     <row r="113">
       <c r="B113" s="6" t="s">
-        <v>2041</v>
+        <v>2103</v>
       </c>
       <c r="C113" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D113" s="6" t="s">
-        <v>2042</v>
+        <v>2104</v>
       </c>
       <c r="E113" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F113" s="6" t="s">
+        <v>2105</v>
+      </c>
     </row>
     <row r="114">
       <c r="B114" s="6" t="s">
-        <v>2043</v>
+        <v>2106</v>
       </c>
       <c r="C114" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D114" s="6" t="s">
-        <v>2044</v>
+        <v>2107</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F114" s="6" t="s">
+        <v>2108</v>
+      </c>
     </row>
     <row r="115">
       <c r="B115" s="6" t="s">
-        <v>2045</v>
+        <v>2109</v>
       </c>
       <c r="C115" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D115" s="6" t="s">
-        <v>2046</v>
+        <v>2110</v>
       </c>
       <c r="E115" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F115" s="6" t="s">
+        <v>2111</v>
+      </c>
     </row>
     <row r="116">
       <c r="B116" s="6" t="s">
-        <v>2047</v>
+        <v>2112</v>
       </c>
       <c r="C116" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D116" s="6" t="s">
-        <v>2048</v>
+        <v>2113</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F116" s="6" t="s">
+        <v>2114</v>
+      </c>
     </row>
     <row r="117">
       <c r="B117" s="6" t="s">
-        <v>2049</v>
+        <v>2115</v>
       </c>
       <c r="C117" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D117" s="6" t="s">
-        <v>2050</v>
+        <v>2116</v>
       </c>
       <c r="E117" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F117" s="6" t="s">
+        <v>2090</v>
+      </c>
     </row>
     <row r="118">
       <c r="B118" s="6" t="s">
-        <v>2051</v>
+        <v>2117</v>
       </c>
       <c r="C118" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D118" s="6" t="s">
-        <v>2052</v>
+        <v>2118</v>
       </c>
       <c r="E118" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F118" s="6" t="s">
+        <v>2099</v>
+      </c>
     </row>
     <row r="119">
       <c r="B119" s="6" t="s">
-        <v>2053</v>
+        <v>2119</v>
       </c>
       <c r="C119" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D119" s="6" t="s">
-        <v>2054</v>
+        <v>2120</v>
       </c>
       <c r="E119" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F119" s="6" t="s">
+        <v>2105</v>
+      </c>
     </row>
     <row r="120">
       <c r="B120" s="6" t="s">
-        <v>2055</v>
+        <v>2121</v>
       </c>
       <c r="C120" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D120" s="6" t="s">
-        <v>2056</v>
+        <v>2122</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>1822</v>
       </c>
+      <c r="F120" s="6" t="s">
+        <v>1878</v>
+      </c>
     </row>
     <row r="121">
       <c r="B121" s="6" t="s">
-        <v>2057</v>
+        <v>2123</v>
       </c>
       <c r="C121" s="6" t="s">
         <v>1821</v>
       </c>
       <c r="D121" s="6" t="s">
-        <v>2058</v>
+        <v>2124</v>
       </c>
       <c r="E121" s="6" t="s">
         <v>1822</v>
+      </c>
+      <c r="F121" s="6" t="s">
+        <v>1844</v>
       </c>
     </row>
   </sheetData>

</xml_diff>